<commit_message>
Br addexamples p sindiv (#50)
*Ajout exemples PS individuel cb22150d7d62887f6af51b9b33fa566751e0eeea
</commit_message>
<xml_diff>
--- a/main/ig/ValueSet-sas-cpts-valueset-typecreneau.xlsx
+++ b/main/ig/ValueSet-sas-cpts-valueset-typecreneau.xlsx
@@ -7,7 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
-    <sheet name="Include from TRE-R314-TypeCre" r:id="rId4" sheetId="2"/>
+    <sheet name="Include from TRE_R314-TypeCre" r:id="rId4" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-18T16:11:48+00:00</t>
+    <t>2024-07-19T13:28:45+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>